<commit_message>
Publish 6/23 rates; hide non-current banks
</commit_message>
<xml_diff>
--- a/rates.xlsx
+++ b/rates.xlsx
@@ -252,6 +252,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>rate-update</author>
+    <author>Rate Update</author>
   </authors>
   <commentList>
     <comment ref="X2" authorId="0" shapeId="0">
@@ -259,86 +260,197 @@
         <t>bankrate.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="Y2" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X3" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; American Express National Bank</t>
       </text>
     </comment>
+    <comment ref="Y3" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+Amex Natl Bank; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="X4" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Online Savings (tiered 3.65% at $0-250k)</t>
       </text>
     </comment>
+    <comment ref="Y4" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X5" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; no rate data on DepositAccounts</t>
       </text>
     </comment>
+    <comment ref="Y5" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X6" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="Y6" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+listed as Alto</t>
+      </text>
+    </comment>
     <comment ref="X7" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Bread Savings; $100 min</t>
       </text>
     </comment>
+    <comment ref="Y7" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1 min</t>
+      </text>
+    </comment>
     <comment ref="X8" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $25 min</t>
       </text>
     </comment>
+    <comment ref="Y8" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$25 min</t>
+      </text>
+    </comment>
     <comment ref="X9" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; 360 Performance Savings</t>
       </text>
     </comment>
+    <comment ref="Y9" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+360 Performance Savings</t>
+      </text>
+    </comment>
     <comment ref="X10" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="Y10" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X11" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; CIBC Bank USA; Agility Savings</t>
       </text>
     </comment>
+    <comment ref="Y11" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X12" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; promo code CITBOOST; base 3.75%, $5,000 min</t>
       </text>
     </comment>
+    <comment ref="Y12" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+Platinum Savings; $5,000 min bal</t>
+      </text>
+    </comment>
     <comment ref="X13" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Citi Accelerate HYS; region-restricted</t>
       </text>
     </comment>
+    <comment ref="Y13" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+Accelerate (region-dependent); not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="X14" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; new accounts only</t>
       </text>
     </comment>
+    <comment ref="Y14" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X15" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; base 3.85%; new-customer boost to 4.15% thru 2026</t>
       </text>
     </comment>
+    <comment ref="Y15" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+4.15% w/ new-customer boost</t>
+      </text>
+    </comment>
     <comment ref="X16" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; LevelUp Savings (top tier may require monthly deposits)</t>
       </text>
     </comment>
+    <comment ref="Y16" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+LevelUp; std req $250/mo deposit</t>
+      </text>
+    </comment>
     <comment ref="X17" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; Personal Savings</t>
       </text>
     </comment>
+    <comment ref="Y17" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X18" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; Marcus by Goldman Sachs</t>
       </text>
     </comment>
+    <comment ref="Y18" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X19" authorId="0" shapeId="0">
       <text>
         <t>not found on either source (as of 2026-06-16)</t>
@@ -354,16 +466,35 @@
         <t>bankrate.com; 2026-06-16; Santander's Openbank; $500 min</t>
       </text>
     </comment>
+    <comment ref="Y21" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X22" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; Envision HYS</t>
       </text>
     </comment>
+    <comment ref="Y22" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X23" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; standard savings; separate HY Savings is region-restricted</t>
       </text>
     </comment>
+    <comment ref="Y23" authorId="1" shapeId="0">
+      <text>
+        <t>Source: pnc.com
+As of: 2026-06-23
+High Yield Savings; eligible markets only</t>
+      </text>
+    </comment>
     <comment ref="X24" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Premier Personal Savings; advertised HYSA not listed as standard</t>
@@ -374,59 +505,134 @@
         <t>bankrate.com; 2026-06-16; Select Savings, new money</t>
       </text>
     </comment>
+    <comment ref="Y25" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X26" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Primis Savings Account, online only</t>
       </text>
     </comment>
+    <comment ref="Y26" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X27" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; High Yield Savings</t>
       </text>
     </comment>
+    <comment ref="Y27" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X28" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="Y28" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="X29" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="Y29" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X30" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; std rate; requires direct deposit (else 0.50%)</t>
       </text>
     </comment>
+    <comment ref="Y30" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+std req direct deposit; 3.10% w/o</t>
+      </text>
+    </comment>
     <comment ref="X31" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="Y31" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X32" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; TAB Bank; High Yield Savings</t>
       </text>
     </comment>
+    <comment ref="Y32" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X33" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Portfolio Savings (3.46% w/ Freedom Checking)</t>
       </text>
     </comment>
+    <comment ref="Y33" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X34" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; base rate; up to ~5% on first $5k w/ qualifying deposits</t>
       </text>
     </comment>
+    <comment ref="Y34" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+5.00% promo on first $5k</t>
+      </text>
+    </comment>
     <comment ref="X35" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="Y35" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="X36" authorId="0" shapeId="0">
       <text>
         <t>bankrate.com; 2026-06-16; via Raisin / Premier</t>
+      </text>
+    </comment>
+    <comment ref="Y36" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
       </text>
     </comment>
   </commentList>
@@ -437,6 +643,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>rate-update</author>
+    <author>Rate Update</author>
   </authors>
   <commentList>
     <comment ref="W2" authorId="0" shapeId="0">
@@ -444,106 +651,249 @@
         <t>depositaccounts.com; 2026-06-16; America First CU; 12-17mo tier; $500 min; membership req</t>
       </text>
     </comment>
+    <comment ref="X2" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
+      </text>
+    </comment>
     <comment ref="W3" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; High Yield CD</t>
       </text>
     </comment>
+    <comment ref="X3" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W4" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X4" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W5" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X5" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
+      </text>
+    </comment>
     <comment ref="W6" authorId="0" shapeId="0">
       <text>
         <t>no rate data on either source (as of 2026-06-16)</t>
       </text>
     </comment>
+    <comment ref="X6" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W7" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X7" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+listed as Alto</t>
+      </text>
+    </comment>
     <comment ref="W8" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,500 min</t>
       </text>
     </comment>
+    <comment ref="X8" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,500 min</t>
+      </text>
+    </comment>
     <comment ref="W9" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; 360 CD</t>
       </text>
     </comment>
+    <comment ref="X9" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W10" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Agility CD; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X10" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W11" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Citizens Access online; $5,000 min</t>
       </text>
     </comment>
+    <comment ref="X11" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+CitizensAccess; $5,000 min</t>
+      </text>
+    </comment>
     <comment ref="W12" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X12" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W13" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X13" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+$500 min; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W14" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X14" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W15" authorId="0" shapeId="0">
       <text>
         <t>not found on either source (as of 2026-06-16)</t>
       </text>
     </comment>
+    <comment ref="X15" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
+      </text>
+    </comment>
     <comment ref="W16" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Online CD (3.75% new money)</t>
       </text>
     </comment>
+    <comment ref="X16" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+Online CD; 3.80% new money; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W17" authorId="0" shapeId="0">
       <text>
         <t>no 12-mo CD listed (only 6-mo) (as of 2026-06-16)</t>
       </text>
     </comment>
+    <comment ref="X17" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W18" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X18" authorId="1" shapeId="0">
+      <text>
+        <t>Source: lendingclub.com
+As of: 2026-06-23
+bank-direct 1yr; eff 6/23/26</t>
+      </text>
+    </comment>
     <comment ref="W19" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X19" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W20" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $2,500 min</t>
       </text>
     </comment>
+    <comment ref="X20" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$2,500 min</t>
+      </text>
+    </comment>
     <comment ref="W21" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X21" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+$500 min; not on Bankrate 1yr</t>
+      </text>
+    </comment>
     <comment ref="W22" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $25,000 min</t>
       </text>
     </comment>
+    <comment ref="X22" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$25,000 min</t>
+      </text>
+    </comment>
     <comment ref="W23" authorId="0" shapeId="0">
       <text>
         <t>not found on either source (as of 2026-06-16)</t>
@@ -554,44 +904,107 @@
         <t>depositaccounts.com; 2026-06-16; $10,000 min</t>
       </text>
     </comment>
+    <comment ref="X24" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+$10,000 min; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W25" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $10,000 min</t>
       </text>
     </comment>
+    <comment ref="X25" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$10,000 min</t>
+      </text>
+    </comment>
     <comment ref="W26" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X26" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
+      </text>
+    </comment>
     <comment ref="W27" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $2,500 min</t>
       </text>
     </comment>
+    <comment ref="X27" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$2,500 min</t>
+      </text>
+    </comment>
     <comment ref="W28" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Share Cert 12-17mo; top tier ($250k); membership req</t>
       </text>
     </comment>
+    <comment ref="X28" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+12-17mo cert; tiered; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W29" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X29" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+std 12mo (13mo promo 4.00%)</t>
+      </text>
+    </comment>
     <comment ref="W30" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; TAB Bank; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X30" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W31" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Union Bank &amp; Trust (NE); $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X31" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+Union Bank &amp; Trust NE; $1,000 min; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W32" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Vio Bank; $500 min</t>
+      </text>
+    </comment>
+    <comment ref="X32" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
       </text>
     </comment>
   </commentList>
@@ -602,6 +1015,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>rate-update</author>
+    <author>Rate Update</author>
   </authors>
   <commentList>
     <comment ref="W2" authorId="0" shapeId="0">
@@ -609,86 +1023,201 @@
         <t>depositaccounts.com; 2026-06-16; America First CU; 24-29mo tier; $500 min; membership req</t>
       </text>
     </comment>
+    <comment ref="X2" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
+      </text>
+    </comment>
     <comment ref="W3" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Raise Your Rate CD</t>
       </text>
     </comment>
+    <comment ref="X3" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W4" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X4" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W5" authorId="0" shapeId="0">
       <text>
         <t>no rate data on either source (as of 2026-06-16)</t>
       </text>
     </comment>
+    <comment ref="X5" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W6" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X6" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+listed as Alto</t>
+      </text>
+    </comment>
     <comment ref="W7" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,500 min</t>
       </text>
     </comment>
+    <comment ref="X7" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,500 min</t>
+      </text>
+    </comment>
     <comment ref="W8" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X8" authorId="1" shapeId="0">
+      <text>
+        <t>Source: capitalone.com
+As of: 2026-06-23
+360 CD 24mo; bank-direct page eff 6/23/26</t>
+      </text>
+    </comment>
     <comment ref="W9" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X9" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W10" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Citizens Access; $5,000 min</t>
       </text>
     </comment>
+    <comment ref="X10" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+CitizensAccess; $5,000 min</t>
+      </text>
+    </comment>
     <comment ref="W11" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X11" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W12" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X12" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+$500 min; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W13" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X13" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W14" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Online CD (3.85% new money)</t>
       </text>
     </comment>
+    <comment ref="X14" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+Online CD; 3.85% new money; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W15" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X15" authorId="1" shapeId="0">
+      <text>
+        <t>Source: lendingclub.com
+As of: 2026-06-23
+bank-direct 2yr; eff 6/23/26</t>
+      </text>
+    </comment>
     <comment ref="W16" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $2,500 min</t>
       </text>
     </comment>
+    <comment ref="X16" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$2,500 min</t>
+      </text>
+    </comment>
     <comment ref="W17" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X17" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W18" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $25,000 min</t>
       </text>
     </comment>
+    <comment ref="X18" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$25,000 min</t>
+      </text>
+    </comment>
     <comment ref="W19" authorId="0" shapeId="0">
       <text>
         <t>not found on either source (as of 2026-06-16)</t>
@@ -699,44 +1228,106 @@
         <t>depositaccounts.com; 2026-06-16; $10,000 min</t>
       </text>
     </comment>
+    <comment ref="X20" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+$10,000 min; not on Bankrate 2yr</t>
+      </text>
+    </comment>
     <comment ref="W21" authorId="0" shapeId="0">
       <text>
         <t>no CDs offered (as of 2026-06-16)</t>
       </text>
     </comment>
+    <comment ref="X21" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W22" authorId="0" shapeId="0">
       <text>
         <t>not found on either source (as of 2026-06-16)</t>
       </text>
     </comment>
+    <comment ref="X22" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+Quorum FCU; $100 min</t>
+      </text>
+    </comment>
     <comment ref="W23" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; 2yr Term CD; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X23" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W24" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $2,500 min</t>
       </text>
     </comment>
+    <comment ref="X24" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$2,500 min</t>
+      </text>
+    </comment>
     <comment ref="W25" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; SchoolsFirst; Share Cert 24-35mo; top tier ($250k); membership req</t>
       </text>
     </comment>
+    <comment ref="X25" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+24-35mo cert; tiered; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W26" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X26" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W27" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; TAB Bank; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X27" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W28" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Vio Bank; $500 min</t>
+      </text>
+    </comment>
+    <comment ref="X28" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
       </text>
     </comment>
   </commentList>
@@ -747,6 +1338,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>rate-update</author>
+    <author>Rate Update</author>
   </authors>
   <commentList>
     <comment ref="W2" authorId="0" shapeId="0">
@@ -754,66 +1346,154 @@
         <t>depositaccounts.com; 2026-06-16; America First CU; 36-47mo tier; $500 min; membership req</t>
       </text>
     </comment>
+    <comment ref="X2" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
+      </text>
+    </comment>
     <comment ref="W3" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; High Yield CD</t>
       </text>
     </comment>
+    <comment ref="X3" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W4" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X4" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W5" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X5" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+listed as Alto</t>
+      </text>
+    </comment>
     <comment ref="W6" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,500 min</t>
       </text>
     </comment>
+    <comment ref="X6" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,500 min</t>
+      </text>
+    </comment>
     <comment ref="W7" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Capital One</t>
       </text>
     </comment>
+    <comment ref="X7" authorId="1" shapeId="0">
+      <text>
+        <t>Source: capitalone.com
+As of: 2026-06-23
+360 CD 36mo; bank-direct page eff 6/23/26</t>
+      </text>
+    </comment>
     <comment ref="W8" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; CFG Bank; $500 min</t>
       </text>
     </comment>
+    <comment ref="X8" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+listed as CFG Bank; $500 min</t>
+      </text>
+    </comment>
     <comment ref="W9" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Citizens Access; $5,000 min</t>
       </text>
     </comment>
+    <comment ref="X9" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+CitizensAccess; $5,000 min</t>
+      </text>
+    </comment>
     <comment ref="W10" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X10" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W11" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X11" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+$500 min; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W12" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X12" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W13" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; First National Bank of America; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X13" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+FNB of America; $1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W14" authorId="0" shapeId="0">
       <text>
         <t>no 36-mo CD listed (as of 2026-06-16)</t>
       </text>
     </comment>
+    <comment ref="X14" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W15" authorId="0" shapeId="0">
       <text>
         <t>no 36-mo CD offered (as of 2026-06-16)</t>
@@ -824,21 +1504,48 @@
         <t>depositaccounts.com; 2026-06-16; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X16" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W17" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $2,500 min</t>
       </text>
     </comment>
+    <comment ref="X17" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$2,500 min</t>
+      </text>
+    </comment>
     <comment ref="W18" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $500 min</t>
       </text>
     </comment>
+    <comment ref="X18" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W19" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $25,000 min</t>
       </text>
     </comment>
+    <comment ref="X19" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$25,000 min</t>
+      </text>
+    </comment>
     <comment ref="W20" authorId="0" shapeId="0">
       <text>
         <t>not found on either source (as of 2026-06-16)</t>
@@ -849,34 +1556,82 @@
         <t>depositaccounts.com; 2026-06-16; $10,000 min</t>
       </text>
     </comment>
+    <comment ref="X21" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$10,000 min</t>
+      </text>
+    </comment>
     <comment ref="W22" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; $2,500 min</t>
       </text>
     </comment>
+    <comment ref="X22" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$2,500 min</t>
+      </text>
+    </comment>
     <comment ref="W23" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Share Cert 36-47mo; top tier ($250k); membership req</t>
       </text>
     </comment>
+    <comment ref="X23" authorId="1" shapeId="0">
+      <text>
+        <t>Source: depositaccounts.com
+As of: 2026-06-23
+36-47mo cert; tiered; not on Bankrate</t>
+      </text>
+    </comment>
     <comment ref="W24" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16</t>
       </text>
     </comment>
+    <comment ref="X24" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23</t>
+      </text>
+    </comment>
     <comment ref="W25" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; TAB Bank; $1,000 min</t>
       </text>
     </comment>
+    <comment ref="X25" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$1,000 min</t>
+      </text>
+    </comment>
     <comment ref="W26" authorId="0" shapeId="0">
       <text>
         <t>depositaccounts.com; 2026-06-16; Vio Bank; $500 min</t>
       </text>
     </comment>
+    <comment ref="X26" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$500 min</t>
+      </text>
+    </comment>
     <comment ref="W27" authorId="0" shapeId="0">
       <text>
         <t>not found on either source (as of 2026-06-16)</t>
+      </text>
+    </comment>
+    <comment ref="X27" authorId="1" shapeId="0">
+      <text>
+        <t>Source: bankrate.com
+As of: 2026-06-23
+$2,500 min</t>
       </text>
     </comment>
   </commentList>
@@ -1184,7 +1939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X44"/>
+  <dimension ref="A1:Y44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14.81640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1278,6 +2033,9 @@
       <c r="X1" s="26" t="n">
         <v>46189</v>
       </c>
+      <c r="Y1" s="26" t="n">
+        <v>46196</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1354,6 +2112,9 @@
       <c r="X2" s="27" t="n">
         <v>0.03</v>
       </c>
+      <c r="Y2" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1424,6 +2185,9 @@
       <c r="X3" s="9" t="n">
         <v>0.031</v>
       </c>
+      <c r="Y3" s="9" t="n">
+        <v>0.031</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1498,6 +2262,9 @@
       <c r="X4" s="27" t="n">
         <v>0.034</v>
       </c>
+      <c r="Y4" s="28" t="n">
+        <v>0.0365</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1574,6 +2341,9 @@
       <c r="X5" s="9" t="n">
         <v>0.0375</v>
       </c>
+      <c r="Y5" s="9" t="n">
+        <v>0.0375</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1650,6 +2420,9 @@
       <c r="X6" s="27" t="n">
         <v>0.03</v>
       </c>
+      <c r="Y6" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1726,6 +2499,9 @@
       <c r="X7" s="9" t="n">
         <v>0.04</v>
       </c>
+      <c r="Y7" s="27" t="n">
+        <v>0.0395</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1802,6 +2578,9 @@
       <c r="X8" s="9" t="n">
         <v>0.0375</v>
       </c>
+      <c r="Y8" s="9" t="n">
+        <v>0.0375</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1873,6 +2652,9 @@
         <v>0.031</v>
       </c>
       <c r="X9" s="27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="Y9" s="9" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -1932,6 +2714,9 @@
       <c r="X10" s="9" t="n">
         <v>0.0325</v>
       </c>
+      <c r="Y10" s="9" t="n">
+        <v>0.0325</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2008,6 +2793,9 @@
       <c r="X11" s="9" t="n">
         <v>0.0352</v>
       </c>
+      <c r="Y11" s="9" t="n">
+        <v>0.0352</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2082,6 +2870,9 @@
         <v>0.041</v>
       </c>
       <c r="X12" s="9" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="Y12" s="9" t="n">
         <v>0.041</v>
       </c>
     </row>
@@ -2141,6 +2932,9 @@
       <c r="X13" s="9" t="n">
         <v>0.031</v>
       </c>
+      <c r="Y13" s="27" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2217,6 +3011,9 @@
       <c r="X14" s="9" t="n">
         <v>0.039</v>
       </c>
+      <c r="Y14" s="9" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2293,6 +3090,9 @@
       <c r="X15" s="9" t="n">
         <v>0.0385</v>
       </c>
+      <c r="Y15" s="9" t="n">
+        <v>0.0385</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2369,6 +3169,9 @@
       <c r="X16" s="9" t="n">
         <v>0.04</v>
       </c>
+      <c r="Y16" s="9" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2445,6 +3248,9 @@
       <c r="X17" s="9" t="n">
         <v>0.038</v>
       </c>
+      <c r="Y17" s="9" t="n">
+        <v>0.038</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2521,6 +3327,9 @@
       <c r="X18" s="27" t="n">
         <v>0.034</v>
       </c>
+      <c r="Y18" s="9" t="n">
+        <v>0.034</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2589,6 +3398,7 @@
         <v>0.039</v>
       </c>
       <c r="X19" s="9" t="n"/>
+      <c r="Y19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -2657,6 +3467,7 @@
         <v>0.0325</v>
       </c>
       <c r="X20" s="9" t="n"/>
+      <c r="Y20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2733,6 +3544,9 @@
       <c r="X21" s="27" t="n">
         <v>0.038</v>
       </c>
+      <c r="Y21" s="9" t="n">
+        <v>0.038</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2807,6 +3621,9 @@
         <v>0.0382</v>
       </c>
       <c r="X22" s="28" t="n">
+        <v>0.0401</v>
+      </c>
+      <c r="Y22" s="9" t="n">
         <v>0.0401</v>
       </c>
     </row>
@@ -2874,6 +3691,9 @@
       <c r="X23" s="27" t="n">
         <v>0.0002</v>
       </c>
+      <c r="Y23" s="28" t="n">
+        <v>0.0315</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2945,6 +3765,7 @@
       <c r="X24" s="27" t="n">
         <v>0.005</v>
       </c>
+      <c r="Y24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3012,6 +3833,9 @@
       <c r="X25" s="9" t="n">
         <v>0.039</v>
       </c>
+      <c r="Y25" s="9" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3085,6 +3909,9 @@
       <c r="X26" s="9" t="n">
         <v>0.0385</v>
       </c>
+      <c r="Y26" s="9" t="n">
+        <v>0.0385</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3155,6 +3982,9 @@
       <c r="X27" s="9" t="n">
         <v>0.032</v>
       </c>
+      <c r="Y27" s="9" t="n">
+        <v>0.032</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3228,6 +4058,9 @@
       <c r="X28" s="9" t="n">
         <v>0.0375</v>
       </c>
+      <c r="Y28" s="9" t="n">
+        <v>0.0375</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3304,6 +4137,9 @@
       <c r="X29" s="9" t="n">
         <v>0.0375</v>
       </c>
+      <c r="Y29" s="9" t="n">
+        <v>0.0375</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3368,6 +4204,9 @@
       <c r="X30" s="28" t="n">
         <v>0.038</v>
       </c>
+      <c r="Y30" s="9" t="n">
+        <v>0.038</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3438,6 +4277,9 @@
       <c r="X31" s="27" t="n">
         <v>0.033</v>
       </c>
+      <c r="Y31" s="9" t="n">
+        <v>0.033</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3514,6 +4356,9 @@
       <c r="X32" s="9" t="n">
         <v>0.0361</v>
       </c>
+      <c r="Y32" s="9" t="n">
+        <v>0.0361</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3590,6 +4435,9 @@
       <c r="X33" s="9" t="n">
         <v>0.0326</v>
       </c>
+      <c r="Y33" s="9" t="n">
+        <v>0.0326</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3664,6 +4512,9 @@
         <v>0.025</v>
       </c>
       <c r="X34" s="9" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="Y34" s="9" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -3737,6 +4588,9 @@
       <c r="X35" s="27" t="n">
         <v>0.0401</v>
       </c>
+      <c r="Y35" s="9" t="n">
+        <v>0.0401</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3805,6 +4659,9 @@
         <v>0.038</v>
       </c>
       <c r="X36" s="9" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="Y36" s="9" t="n">
         <v>0.038</v>
       </c>
     </row>
@@ -3938,6 +4795,9 @@
       <c r="W1" s="26" t="n">
         <v>46189</v>
       </c>
+      <c r="X1" s="26" t="n">
+        <v>46196</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4009,6 +4869,9 @@
       <c r="W2" s="9" t="n">
         <v>0.0395</v>
       </c>
+      <c r="X2" s="9" t="n">
+        <v>0.0395</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4082,6 +4945,9 @@
       <c r="W3" s="9" t="n">
         <v>0.037</v>
       </c>
+      <c r="X3" s="9" t="n">
+        <v>0.037</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4152,6 +5018,9 @@
       <c r="W4" s="9" t="n">
         <v>0.0325</v>
       </c>
+      <c r="X4" s="9" t="n">
+        <v>0.0325</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4219,6 +5088,9 @@
       <c r="W5" s="9" t="n">
         <v>0.032</v>
       </c>
+      <c r="X5" s="9" t="n">
+        <v>0.032</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4290,6 +5162,9 @@
         <v>0.0405</v>
       </c>
       <c r="W6" s="9" t="n"/>
+      <c r="X6" s="9" t="n">
+        <v>0.041</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4363,6 +5238,9 @@
       <c r="W7" s="9" t="n">
         <v>0.025</v>
       </c>
+      <c r="X7" s="9" t="n">
+        <v>0.025</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4436,6 +5314,9 @@
       <c r="W8" s="28" t="n">
         <v>0.04</v>
       </c>
+      <c r="X8" s="9" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4506,6 +5387,9 @@
       <c r="W9" s="9" t="n">
         <v>0.039</v>
       </c>
+      <c r="X9" s="9" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4577,6 +5461,9 @@
         <v>0.04</v>
       </c>
       <c r="W10" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="X10" s="9" t="n">
         <v>0.04</v>
       </c>
     </row>
@@ -4650,6 +5537,9 @@
       <c r="W11" s="9" t="n">
         <v>0.0325</v>
       </c>
+      <c r="X11" s="9" t="n">
+        <v>0.0325</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4721,6 +5611,9 @@
         <v>0.034</v>
       </c>
       <c r="W12" s="9" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="X12" s="9" t="n">
         <v>0.034</v>
       </c>
     </row>
@@ -4769,6 +5662,9 @@
       <c r="W13" s="27" t="n">
         <v>0.0385</v>
       </c>
+      <c r="X13" s="9" t="n">
+        <v>0.0385</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4842,6 +5738,9 @@
       <c r="W14" s="9" t="n">
         <v>0.0367</v>
       </c>
+      <c r="X14" s="9" t="n">
+        <v>0.0367</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4913,7 +5812,9 @@
         <v>0.0356</v>
       </c>
       <c r="W15" s="9" t="n"/>
-      <c r="X15" s="9" t="n"/>
+      <c r="X15" s="9" t="n">
+        <v>0.0356</v>
+      </c>
       <c r="Y15" s="9" t="n"/>
       <c r="Z15" s="9" t="n"/>
     </row>
@@ -4970,6 +5871,9 @@
       </c>
       <c r="W16" s="28" t="n">
         <v>0.037</v>
+      </c>
+      <c r="X16" s="28" t="n">
+        <v>0.0375</v>
       </c>
     </row>
     <row r="17">
@@ -5032,6 +5936,9 @@
         <v>0.0015</v>
       </c>
       <c r="W17" s="9" t="n"/>
+      <c r="X17" s="9" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5102,6 +6009,9 @@
       <c r="W18" s="9" t="n">
         <v>0.035</v>
       </c>
+      <c r="X18" s="9" t="n">
+        <v>0.035</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5173,6 +6083,9 @@
         <v>0.0403</v>
       </c>
       <c r="W19" s="28" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="X19" s="9" t="n">
         <v>0.041</v>
       </c>
     </row>
@@ -5246,6 +6159,9 @@
       <c r="W20" s="27" t="n">
         <v>0.039</v>
       </c>
+      <c r="X20" s="28" t="n">
+        <v>0.041</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5316,6 +6232,9 @@
       <c r="W21" s="9" t="n">
         <v>0.039</v>
       </c>
+      <c r="X21" s="9" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5387,6 +6306,9 @@
         <v>0.0405</v>
       </c>
       <c r="W22" s="28" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="X22" s="9" t="n">
         <v>0.041</v>
       </c>
     </row>
@@ -5454,6 +6376,7 @@
         <v>0.0305</v>
       </c>
       <c r="W23" s="9" t="n"/>
+      <c r="X23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5520,6 +6443,9 @@
         <v>0.0395</v>
       </c>
       <c r="W24" s="9" t="n">
+        <v>0.0395</v>
+      </c>
+      <c r="X24" s="9" t="n">
         <v>0.0395</v>
       </c>
     </row>
@@ -5585,6 +6511,9 @@
       <c r="W25" s="28" t="n">
         <v>0.0415</v>
       </c>
+      <c r="X25" s="9" t="n">
+        <v>0.0415</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5649,6 +6578,9 @@
       <c r="W26" s="9" t="n">
         <v>0.03</v>
       </c>
+      <c r="X26" s="28" t="n">
+        <v>0.035</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5721,6 +6653,9 @@
       </c>
       <c r="W27" s="9" t="n">
         <v>0.038</v>
+      </c>
+      <c r="X27" s="28" t="n">
+        <v>0.039</v>
       </c>
     </row>
     <row r="28">
@@ -5778,6 +6713,9 @@
       <c r="W28" s="28" t="n">
         <v>0.0395</v>
       </c>
+      <c r="X28" s="9" t="n">
+        <v>0.0395</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5836,6 +6774,9 @@
       <c r="W29" s="9" t="n">
         <v>0.037</v>
       </c>
+      <c r="X29" s="9" t="n">
+        <v>0.037</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5909,6 +6850,9 @@
       <c r="W30" s="28" t="n">
         <v>0.04</v>
       </c>
+      <c r="X30" s="9" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5973,6 +6917,9 @@
       <c r="W31" s="28" t="n">
         <v>0.0375</v>
       </c>
+      <c r="X31" s="28" t="n">
+        <v>0.0385</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6044,6 +6991,9 @@
         <v>0.038</v>
       </c>
       <c r="W32" s="9" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="X32" s="9" t="n">
         <v>0.038</v>
       </c>
     </row>
@@ -6094,7 +7044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W34"/>
+  <dimension ref="A1:X34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6183,6 +7133,9 @@
       <c r="W1" s="26" t="n">
         <v>46189</v>
       </c>
+      <c r="X1" s="26" t="n">
+        <v>46196</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6252,6 +7205,9 @@
       </c>
       <c r="W2" s="9" t="n">
         <v>0.0405</v>
+      </c>
+      <c r="X2" s="28" t="n">
+        <v>0.041</v>
       </c>
     </row>
     <row r="3">
@@ -6322,6 +7278,9 @@
       <c r="W3" s="9" t="n">
         <v>0.03</v>
       </c>
+      <c r="X3" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6392,6 +7351,9 @@
       <c r="W4" s="9" t="n">
         <v>0.03</v>
       </c>
+      <c r="X4" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6463,6 +7425,9 @@
         <v>0.0365</v>
       </c>
       <c r="W5" s="9" t="n"/>
+      <c r="X5" s="9" t="n">
+        <v>0.0365</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6536,6 +7501,9 @@
       <c r="W6" s="28" t="n">
         <v>0.0255</v>
       </c>
+      <c r="X6" s="9" t="n">
+        <v>0.0255</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6609,6 +7577,9 @@
       <c r="W7" s="28" t="n">
         <v>0.04</v>
       </c>
+      <c r="X7" s="9" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6679,6 +7650,9 @@
       <c r="W8" s="9" t="n">
         <v>0.035</v>
       </c>
+      <c r="X8" s="9" t="n">
+        <v>0.035</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6752,6 +7726,9 @@
       <c r="W9" s="27" t="n">
         <v>0.03</v>
       </c>
+      <c r="X9" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6823,6 +7800,9 @@
       <c r="W10" s="9" t="n">
         <v>0.03</v>
       </c>
+      <c r="X10" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6896,6 +7876,9 @@
       <c r="W11" s="9" t="n">
         <v>0.034</v>
       </c>
+      <c r="X11" s="9" t="n">
+        <v>0.034</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6951,6 +7934,9 @@
       <c r="W12" s="9" t="n">
         <v>0.0384</v>
       </c>
+      <c r="X12" s="9" t="n">
+        <v>0.0384</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7022,6 +8008,9 @@
         <v>0.033</v>
       </c>
       <c r="W13" s="9" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="X13" s="9" t="n">
         <v>0.033</v>
       </c>
     </row>
@@ -7078,6 +8067,9 @@
       <c r="W14" s="28" t="n">
         <v>0.038</v>
       </c>
+      <c r="X14" s="9" t="n">
+        <v>0.038</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7149,6 +8141,9 @@
       <c r="W15" s="9" t="n">
         <v>0.035</v>
       </c>
+      <c r="X15" s="9" t="n">
+        <v>0.035</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7220,6 +8215,9 @@
         <v>0.02</v>
       </c>
       <c r="W16" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="X16" s="9" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -7290,6 +8288,9 @@
       <c r="W17" s="9" t="n">
         <v>0.037</v>
       </c>
+      <c r="X17" s="9" t="n">
+        <v>0.037</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7361,6 +8362,9 @@
         <v>0.0415</v>
       </c>
       <c r="W18" s="28" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="X18" s="9" t="n">
         <v>0.042</v>
       </c>
     </row>
@@ -7428,6 +8432,7 @@
         <v>0.0285</v>
       </c>
       <c r="W19" s="9" t="n"/>
+      <c r="X19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7494,6 +8499,9 @@
         <v>0.0385</v>
       </c>
       <c r="W20" s="9" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="X20" s="9" t="n">
         <v>0.0385</v>
       </c>
     </row>
@@ -7555,6 +8563,9 @@
         <v>0.0169</v>
       </c>
       <c r="W21" s="9" t="n"/>
+      <c r="X21" s="9" t="n">
+        <v>0.0169</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7626,6 +8637,9 @@
         <v>0.03</v>
       </c>
       <c r="W22" s="9" t="n"/>
+      <c r="X22" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7696,6 +8710,9 @@
       <c r="W23" s="28" t="n">
         <v>0.03</v>
       </c>
+      <c r="X23" s="9" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7767,6 +8784,9 @@
         <v>0.0385</v>
       </c>
       <c r="W24" s="9" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="X24" s="9" t="n">
         <v>0.0385</v>
       </c>
     </row>
@@ -7823,6 +8843,9 @@
       <c r="W25" s="28" t="n">
         <v>0.04</v>
       </c>
+      <c r="X25" s="9" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7881,6 +8904,9 @@
       <c r="W26" s="9" t="n">
         <v>0.035</v>
       </c>
+      <c r="X26" s="9" t="n">
+        <v>0.035</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7954,6 +8980,9 @@
       <c r="W27" s="28" t="n">
         <v>0.041</v>
       </c>
+      <c r="X27" s="9" t="n">
+        <v>0.041</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8025,6 +9054,9 @@
         <v>0.035</v>
       </c>
       <c r="W28" s="9" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="X28" s="9" t="n">
         <v>0.035</v>
       </c>
     </row>
@@ -8063,7 +9095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W34"/>
+  <dimension ref="A1:X34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="17.26953125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8158,6 +9190,9 @@
       <c r="W1" s="26" t="n">
         <v>46189</v>
       </c>
+      <c r="X1" s="26" t="n">
+        <v>46196</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8228,6 +9263,9 @@
       <c r="W2" s="9" t="n">
         <v>0.0405</v>
       </c>
+      <c r="X2" s="9" t="n">
+        <v>0.0405</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8297,6 +9335,9 @@
         <v>0.034</v>
       </c>
       <c r="W3" s="9" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="X3" s="9" t="n">
         <v>0.034</v>
       </c>
     </row>
@@ -8365,6 +9406,9 @@
       <c r="W4" s="9" t="n">
         <v>0.0225</v>
       </c>
+      <c r="X4" s="9" t="n">
+        <v>0.0225</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8438,6 +9482,9 @@
       <c r="W5" s="28" t="n">
         <v>0.026</v>
       </c>
+      <c r="X5" s="9" t="n">
+        <v>0.026</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8511,6 +9558,9 @@
       <c r="W6" s="28" t="n">
         <v>0.04</v>
       </c>
+      <c r="X6" s="9" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8579,6 +9629,9 @@
         <v>0.035</v>
       </c>
       <c r="W7" s="9" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="X7" s="9" t="n">
         <v>0.035</v>
       </c>
     </row>
@@ -8640,6 +9693,9 @@
       <c r="W8" s="9" t="n">
         <v>0.0335</v>
       </c>
+      <c r="X8" s="9" t="n">
+        <v>0.0335</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8708,6 +9764,9 @@
       <c r="W9" s="9" t="n">
         <v>0.0275</v>
       </c>
+      <c r="X9" s="9" t="n">
+        <v>0.0275</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8779,6 +9838,9 @@
         <v>0.034</v>
       </c>
       <c r="W10" s="9" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="X10" s="9" t="n">
         <v>0.034</v>
       </c>
     </row>
@@ -8830,6 +9892,9 @@
       <c r="W11" s="9" t="n">
         <v>0.0384</v>
       </c>
+      <c r="X11" s="9" t="n">
+        <v>0.0384</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8901,6 +9966,9 @@
         <v>0.033</v>
       </c>
       <c r="W12" s="9" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="X12" s="9" t="n">
         <v>0.033</v>
       </c>
     </row>
@@ -8961,6 +10029,9 @@
       <c r="W13" s="9" t="n">
         <v>0.038</v>
       </c>
+      <c r="X13" s="28" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9029,6 +10100,9 @@
         <v>0.0015</v>
       </c>
       <c r="W14" s="9" t="n"/>
+      <c r="X14" s="9" t="n">
+        <v>0.0015</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9086,6 +10160,7 @@
         <v>0.0345</v>
       </c>
       <c r="W15" s="9" t="n"/>
+      <c r="X15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9156,6 +10231,9 @@
       <c r="W16" s="9" t="n">
         <v>0.0365</v>
       </c>
+      <c r="X16" s="9" t="n">
+        <v>0.0365</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9227,6 +10305,9 @@
         <v>0.02</v>
       </c>
       <c r="W17" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="X17" s="9" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -9300,6 +10381,9 @@
       <c r="W18" s="9" t="n">
         <v>0.037</v>
       </c>
+      <c r="X18" s="9" t="n">
+        <v>0.037</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9369,6 +10453,9 @@
         <v>0.0415</v>
       </c>
       <c r="W19" s="28" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="X19" s="9" t="n">
         <v>0.042</v>
       </c>
     </row>
@@ -9436,6 +10523,7 @@
         <v>0.0285</v>
       </c>
       <c r="W20" s="9" t="n"/>
+      <c r="X20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9507,6 +10595,9 @@
         <v>0.0385</v>
       </c>
       <c r="W21" s="9" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="X21" s="9" t="n">
         <v>0.0385</v>
       </c>
     </row>
@@ -9579,6 +10670,9 @@
       </c>
       <c r="W22" s="9" t="n">
         <v>0.0395</v>
+      </c>
+      <c r="X22" s="28" t="n">
+        <v>0.0405</v>
       </c>
     </row>
     <row r="23">
@@ -9637,6 +10731,9 @@
       <c r="W23" s="28" t="n">
         <v>0.04</v>
       </c>
+      <c r="X23" s="9" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9698,6 +10795,9 @@
       <c r="W24" s="9" t="n">
         <v>0.036</v>
       </c>
+      <c r="X24" s="9" t="n">
+        <v>0.036</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9771,6 +10871,9 @@
       <c r="W25" s="28" t="n">
         <v>0.0415</v>
       </c>
+      <c r="X25" s="9" t="n">
+        <v>0.0415</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9842,6 +10945,9 @@
         <v>0.035</v>
       </c>
       <c r="W26" s="9" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="X26" s="9" t="n">
         <v>0.035</v>
       </c>
     </row>
@@ -9905,6 +11011,9 @@
         <v>0.0025</v>
       </c>
       <c r="W27" s="9" t="n"/>
+      <c r="X27" s="9" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="1" t="n"/>

</xml_diff>